<commit_message>
chore: update Matriz.xlsx with new data
</commit_message>
<xml_diff>
--- a/docs/Matriz.xlsx
+++ b/docs/Matriz.xlsx
@@ -6127,7 +6127,7 @@
     <row r="1" ht="26.15" customHeight="1" s="45">
       <c r="A1" s="46" t="inlineStr">
         <is>
-          <t>M4 · MATRIZ DE PRUEBA DE ESTRÉS · clasedominio</t>
+          <t>M4 · MATRIZ DE PRUEBA DE ESTRÉS · portfolio (codebymike.tech)</t>
         </is>
       </c>
     </row>
@@ -6139,7 +6139,7 @@
       </c>
       <c r="B3" s="10" t="inlineStr">
         <is>
-          <t>http://localhost:8080</t>
+          <t>http://127.0.0.1:4400 (npm run dev:carga)</t>
         </is>
       </c>
       <c r="D3" s="9" t="inlineStr">
@@ -6149,7 +6149,7 @@
       </c>
       <c r="E3" s="10" t="inlineStr">
         <is>
-          <t>Apache JMeter 5.6.3</t>
+          <t>Apache k6 · lab/k6/estres.js</t>
         </is>
       </c>
     </row>
@@ -6159,10 +6159,14 @@
           <t>Entorno:</t>
         </is>
       </c>
-      <c r="B4" s="10" t="n"/>
+      <c r="B4" s="10" t="inlineStr">
+        <is>
+          <t>Node 22.22.3 · Astro 7 dev · sqld local (Turso) en Docker · host descontendido (11 contenedores ajenos detenidos)</t>
+        </is>
+      </c>
       <c r="D4" s="9" t="inlineStr">
         <is>
-          <t>Fecha:</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="E4" s="10" t="n"/>
@@ -6175,7 +6179,7 @@
       </c>
       <c r="B5" s="10" t="inlineStr">
         <is>
-          <t>Punto de saturación, punto de quiebre y recuperación</t>
+          <t>Punto de saturación, punto de quiebre y recuperación, vía ramping-arrival-rate 50→300 req/s en escalones de 30s + recuperación de 120s a 100 req/s</t>
         </is>
       </c>
       <c r="D5" s="9" t="inlineStr">
@@ -6183,12 +6187,16 @@
           <t>Responsable:</t>
         </is>
       </c>
-      <c r="E5" s="10" t="n"/>
+      <c r="E5" s="10" t="inlineStr">
+        <is>
+          <t>Mike (@mikerb95)</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="26.15" customHeight="1" s="45">
       <c r="A6" s="52" t="inlineStr">
         <is>
-          <t>Nota · Ejemplo de hallazgo: "El throughput se estanca en 250 req/s desde 400 usuarios mientras la CPU llega al 97 %". Recomendacion: ampliar el pool de conexiones con spring.datasource.hikari.maximum-pool-size.</t>
+          <t>Nota · A diferencia de la plantilla original (VUs fijos), este script controla el RITMO DE LLEGADA (ramping-arrival-rate, req/s ofrecidos), no la concurrencia: con VUs, el sistema se autoprotege bajando la carga cuando se satura y nunca se encuentra el punto de quiebre. La columna "Usuarios" muestra los VUs promedio que k6 tuvo que asignar para sostener ese ritmo (a más saturación, más VUs para la misma tasa de llegada). Fuente: lab/k6/resultados/estres-2026-08-27T15-10-31-684Z.json.</t>
         </is>
       </c>
       <c r="B6" s="55" t="n"/>
@@ -6254,44 +6262,16 @@
       </c>
     </row>
     <row r="8" ht="30" customHeight="1" s="45">
-      <c r="A8" s="12" t="inlineStr">
-        <is>
-          <t>E0</t>
-        </is>
-      </c>
-      <c r="B8" s="12" t="n">
-        <v>25</v>
-      </c>
-      <c r="C8" s="12" t="inlineStr">
-        <is>
-          <t>3 min</t>
-        </is>
-      </c>
-      <c r="D8" s="12" t="n">
-        <v>24</v>
-      </c>
-      <c r="E8" s="23" t="n">
-        <v>180</v>
-      </c>
-      <c r="F8" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="G8" s="12" t="n">
-        <v>22</v>
-      </c>
-      <c r="H8" s="12" t="n">
-        <v>34</v>
-      </c>
-      <c r="I8" s="13" t="inlineStr">
-        <is>
-          <t>EJEMPLO · Borre esta fila</t>
-        </is>
-      </c>
-      <c r="J8" s="12" t="inlineStr">
-        <is>
-          <t>APROBADA</t>
-        </is>
-      </c>
+      <c r="A8" s="12" t="n"/>
+      <c r="B8" s="12" t="n"/>
+      <c r="C8" s="12" t="n"/>
+      <c r="D8" s="12" t="n"/>
+      <c r="E8" s="23" t="n"/>
+      <c r="F8" s="24" t="n"/>
+      <c r="G8" s="12" t="n"/>
+      <c r="H8" s="12" t="n"/>
+      <c r="I8" s="13" t="n"/>
+      <c r="J8" s="12" t="n"/>
     </row>
     <row r="9" ht="30" customHeight="1" s="45">
       <c r="A9" s="14" t="inlineStr">
@@ -6300,24 +6280,40 @@
         </is>
       </c>
       <c r="B9" s="14" t="n">
-        <v>25</v>
+        <v>12</v>
       </c>
       <c r="C9" s="14" t="inlineStr">
         <is>
-          <t>3 min</t>
-        </is>
-      </c>
-      <c r="D9" s="25" t="n"/>
-      <c r="E9" s="26" t="n"/>
-      <c r="F9" s="27" t="n"/>
-      <c r="G9" s="25" t="n"/>
-      <c r="H9" s="25" t="n"/>
+          <t>30 s</t>
+        </is>
+      </c>
+      <c r="D9" s="25" t="n">
+        <v>49.9</v>
+      </c>
+      <c r="E9" s="26" t="n">
+        <v>1282</v>
+      </c>
+      <c r="F9" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="G9" s="25" t="n">
+        <v>14</v>
+      </c>
+      <c r="H9" s="25" t="inlineStr">
+        <is>
+          <t>308 MB</t>
+        </is>
+      </c>
       <c r="I9" s="15" t="inlineStr">
         <is>
-          <t>Línea base de comparación</t>
-        </is>
-      </c>
-      <c r="J9" s="16" t="n"/>
+          <t>Escalón sano (50 req/s ofrecidos): línea base de comparación.</t>
+        </is>
+      </c>
+      <c r="J9" s="16" t="inlineStr">
+        <is>
+          <t>APROBADA</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="30" customHeight="1" s="45">
       <c r="A10" s="17" t="inlineStr">
@@ -6326,20 +6322,40 @@
         </is>
       </c>
       <c r="B10" s="17" t="n">
-        <v>50</v>
+        <v>184</v>
       </c>
       <c r="C10" s="17" t="inlineStr">
         <is>
-          <t>3 min</t>
-        </is>
-      </c>
-      <c r="D10" s="28" t="n"/>
-      <c r="E10" s="29" t="n"/>
-      <c r="F10" s="30" t="n"/>
-      <c r="G10" s="28" t="n"/>
-      <c r="H10" s="28" t="n"/>
-      <c r="I10" s="18" t="n"/>
-      <c r="J10" s="53" t="n"/>
+          <t>30 s</t>
+        </is>
+      </c>
+      <c r="D10" s="28" t="n">
+        <v>69.8</v>
+      </c>
+      <c r="E10" s="29" t="n">
+        <v>7938.9</v>
+      </c>
+      <c r="F10" s="30" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="G10" s="28" t="n">
+        <v>14.8</v>
+      </c>
+      <c r="H10" s="28" t="inlineStr">
+        <is>
+          <t>354 MB</t>
+        </is>
+      </c>
+      <c r="I10" s="18" t="inlineStr">
+        <is>
+          <t>Primer escalón degradado (100 req/s ofrecidos): el throughput ya no sigue al ritmo ofrecido y el p95 se dispara.</t>
+        </is>
+      </c>
+      <c r="J10" s="53" t="inlineStr">
+        <is>
+          <t>OBSERVACION</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="30" customHeight="1" s="45">
       <c r="A11" s="14" t="inlineStr">
@@ -6348,24 +6364,40 @@
         </is>
       </c>
       <c r="B11" s="14" t="n">
-        <v>100</v>
+        <v>1228</v>
       </c>
       <c r="C11" s="14" t="inlineStr">
         <is>
-          <t>3 min</t>
-        </is>
-      </c>
-      <c r="D11" s="25" t="n"/>
-      <c r="E11" s="26" t="n"/>
-      <c r="F11" s="27" t="n"/>
-      <c r="G11" s="25" t="n"/>
-      <c r="H11" s="25" t="n"/>
+          <t>30 s</t>
+        </is>
+      </c>
+      <c r="D11" s="25" t="n">
+        <v>27.1</v>
+      </c>
+      <c r="E11" s="26" t="n">
+        <v>10001</v>
+      </c>
+      <c r="F11" s="27" t="n">
+        <v>76.3</v>
+      </c>
+      <c r="G11" s="25" t="n">
+        <v>16.4</v>
+      </c>
+      <c r="H11" s="25" t="inlineStr">
+        <is>
+          <t>355 MB</t>
+        </is>
+      </c>
       <c r="I11" s="15" t="inlineStr">
         <is>
-          <t>Carga objetivo: aquí deben cumplirse los umbrales</t>
-        </is>
-      </c>
-      <c r="J11" s="16" t="n"/>
+          <t>¿Punto de quiebre? (200 req/s ofrecidos): la mayoría de peticiones agotan el timeout de 10s. H-01.</t>
+        </is>
+      </c>
+      <c r="J11" s="16" t="inlineStr">
+        <is>
+          <t>FALLIDA</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="30" customHeight="1" s="45">
       <c r="A12" s="17" t="inlineStr">
@@ -6374,20 +6406,42 @@
         </is>
       </c>
       <c r="B12" s="17" t="n">
-        <v>200</v>
+        <v>2330</v>
       </c>
       <c r="C12" s="17" t="inlineStr">
         <is>
-          <t>3 min</t>
-        </is>
-      </c>
-      <c r="D12" s="28" t="n"/>
-      <c r="E12" s="29" t="n"/>
-      <c r="F12" s="30" t="n"/>
-      <c r="G12" s="28" t="n"/>
-      <c r="H12" s="28" t="n"/>
-      <c r="I12" s="18" t="n"/>
-      <c r="J12" s="53" t="n"/>
+          <t>30 s</t>
+        </is>
+      </c>
+      <c r="D12" s="28" t="n">
+        <v>0</v>
+      </c>
+      <c r="E12" s="29" t="n">
+        <v>10000.8</v>
+      </c>
+      <c r="F12" s="30" t="n">
+        <v>100</v>
+      </c>
+      <c r="G12" s="28" t="inlineStr">
+        <is>
+          <t>s/d</t>
+        </is>
+      </c>
+      <c r="H12" s="28" t="inlineStr">
+        <is>
+          <t>s/d</t>
+        </is>
+      </c>
+      <c r="I12" s="18" t="inlineStr">
+        <is>
+          <t>300 req/s ofrecidos, primera ventana: 100% de error. CPU/heap sin dato porque el propio endpoint de diagnóstico también se satura (H-04).</t>
+        </is>
+      </c>
+      <c r="J12" s="53" t="inlineStr">
+        <is>
+          <t>FALLIDA</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="30" customHeight="1" s="45">
       <c r="A13" s="14" t="inlineStr">
@@ -6396,24 +6450,42 @@
         </is>
       </c>
       <c r="B13" s="14" t="n">
-        <v>400</v>
+        <v>2852</v>
       </c>
       <c r="C13" s="14" t="inlineStr">
         <is>
-          <t>3 min</t>
-        </is>
-      </c>
-      <c r="D13" s="25" t="n"/>
-      <c r="E13" s="26" t="n"/>
-      <c r="F13" s="27" t="n"/>
-      <c r="G13" s="25" t="n"/>
-      <c r="H13" s="25" t="n"/>
+          <t>30 s</t>
+        </is>
+      </c>
+      <c r="D13" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="E13" s="26" t="n">
+        <v>10000.4</v>
+      </c>
+      <c r="F13" s="27" t="n">
+        <v>100</v>
+      </c>
+      <c r="G13" s="25" t="inlineStr">
+        <is>
+          <t>s/d</t>
+        </is>
+      </c>
+      <c r="H13" s="25" t="inlineStr">
+        <is>
+          <t>s/d</t>
+        </is>
+      </c>
       <c r="I13" s="15" t="inlineStr">
         <is>
-          <t>¿Punto de saturación? El throughput deja de crecer</t>
-        </is>
-      </c>
-      <c r="J13" s="16" t="n"/>
+          <t>300 req/s ofrecidos, segunda ventana: el colapso se sostiene, hasta 2930 VUs simultáneos asignados por k6.</t>
+        </is>
+      </c>
+      <c r="J13" s="16" t="inlineStr">
+        <is>
+          <t>FALLIDA</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="30" customHeight="1" s="45">
       <c r="A14" s="17" t="inlineStr">
@@ -6436,10 +6508,14 @@
       <c r="H14" s="28" t="n"/>
       <c r="I14" s="18" t="inlineStr">
         <is>
-          <t>¿Punto de quiebre? Aparecen errores y timeouts</t>
-        </is>
-      </c>
-      <c r="J14" s="53" t="n"/>
+          <t>No se ejecutó: el escalón anterior ya estaba en 100% de error; ampliar el ritmo no habría añadido información (ver diseño en lab/k6/estres.js).</t>
+        </is>
+      </c>
+      <c r="J14" s="53" t="inlineStr">
+        <is>
+          <t>BLOQUEADA</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="30" customHeight="1" s="45">
       <c r="A15" s="14" t="inlineStr">
@@ -6452,20 +6528,40 @@
       </c>
       <c r="C15" s="14" t="inlineStr">
         <is>
-          <t>5 min</t>
+          <t>120 s (8 tramos de 15 s)</t>
         </is>
       </c>
       <c r="D15" s="25" t="n"/>
-      <c r="E15" s="26" t="n"/>
-      <c r="F15" s="27" t="n"/>
-      <c r="G15" s="25" t="n"/>
-      <c r="H15" s="25" t="n"/>
+      <c r="E15" s="26" t="inlineStr">
+        <is>
+          <t>10000.6 (agregado) / 60.4 (tramo final)</t>
+        </is>
+      </c>
+      <c r="F15" s="27" t="inlineStr">
+        <is>
+          <t>27.1 (agregado)</t>
+        </is>
+      </c>
+      <c r="G15" s="25" t="inlineStr">
+        <is>
+          <t>6.1–16.1</t>
+        </is>
+      </c>
+      <c r="H15" s="25" t="inlineStr">
+        <is>
+          <t>224–368 MB</t>
+        </is>
+      </c>
       <c r="I15" s="15" t="inlineStr">
         <is>
-          <t>Recuperación: tiempo hasta volver a los valores de E3</t>
-        </is>
-      </c>
-      <c r="J15" s="16" t="n"/>
+          <t>Agregado engañoso: los primeros 45s siguen saturados (p95≈10000ms); recién desde +75s converge (p50 24–26ms, p95 60–63ms), MEJOR que el propio E1. Recupera del todo pero no de inmediato: tarda ~75s en iniciar. H-02, H-03.</t>
+        </is>
+      </c>
+      <c r="J15" s="16" t="inlineStr">
+        <is>
+          <t>OBSERVACION</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="30" customHeight="1" s="45">
       <c r="A16" s="18" t="n"/>
@@ -6516,11 +6612,19 @@
           <t>H-01</t>
         </is>
       </c>
-      <c r="B21" s="53" t="n"/>
+      <c r="B21" s="53" t="inlineStr">
+        <is>
+          <t>Host limpio: el punto de quiebre vuelve a ~100 req/s (11 contenedores ajenos detenidos, load average 2.19→0.37-0.98). El escalón de 50 req/s vuelve a 0% de error, igual que la corrida sin contención del 22 ago.</t>
+        </is>
+      </c>
       <c r="C21" s="55" t="n"/>
       <c r="D21" s="55" t="n"/>
       <c r="E21" s="56" t="n"/>
-      <c r="F21" s="53" t="n"/>
+      <c r="F21" s="53" t="inlineStr">
+        <is>
+          <t>Repetir corridas de estrés siempre con el host descontendido; documentar la carga ambiental como variable de la prueba.</t>
+        </is>
+      </c>
       <c r="G21" s="55" t="n"/>
       <c r="H21" s="55" t="n"/>
       <c r="I21" s="55" t="n"/>
@@ -6532,11 +6636,19 @@
           <t>H-02</t>
         </is>
       </c>
-      <c r="B22" s="53" t="n"/>
+      <c r="B22" s="53" t="inlineStr">
+        <is>
+          <t>El agregado de la fase de recuperación (120s) da 27.1% de error y p95≈10000ms, pero por tramos de 15s se ve que converge del todo desde +75-90s (p50 24-26ms), mejor que el propio escalón sano E1.</t>
+        </is>
+      </c>
       <c r="C22" s="55" t="n"/>
       <c r="D22" s="55" t="n"/>
       <c r="E22" s="56" t="n"/>
-      <c r="F22" s="53" t="n"/>
+      <c r="F22" s="53" t="inlineStr">
+        <is>
+          <t>Medir siempre la recuperación por tramos, no en agregado: el agregado esconde una recuperación completa detrás de la cola inicial que aún drena.</t>
+        </is>
+      </c>
       <c r="G22" s="55" t="n"/>
       <c r="H22" s="55" t="n"/>
       <c r="I22" s="55" t="n"/>
@@ -6548,11 +6660,19 @@
           <t>H-03</t>
         </is>
       </c>
-      <c r="B23" s="53" t="n"/>
+      <c r="B23" s="53" t="inlineStr">
+        <is>
+          <t>El drenaje de ~60-75s tras cortar la carga no es contención de host: coincide con las ~2930 conexiones simultáneas que dejó el último escalón (300 req/s, 100% error, corte en seco con gracefulStop:"0s").</t>
+        </is>
+      </c>
       <c r="C23" s="55" t="n"/>
       <c r="D23" s="55" t="n"/>
       <c r="E23" s="56" t="n"/>
-      <c r="F23" s="53" t="n"/>
+      <c r="F23" s="53" t="inlineStr">
+        <is>
+          <t>El límite real parece ser la concurrencia de sockets/handlers de `astro dev`, no CPU/memoria; repetir contra un build de producción (astro build + preview, o Vercel) antes de fijar un SLO de capacidad.</t>
+        </is>
+      </c>
       <c r="G23" s="55" t="n"/>
       <c r="H23" s="55" t="n"/>
       <c r="I23" s="55" t="n"/>
@@ -6564,11 +6684,19 @@
           <t>H-04</t>
         </is>
       </c>
-      <c r="B24" s="53" t="n"/>
+      <c r="B24" s="53" t="inlineStr">
+        <is>
+          <t>cpuPct/heapMb quedan sin dato en los 2 últimos escalones (300 req/s) y en los primeros 45s de recuperación: el propio endpoint de diagnóstico /api/lab/proceso también se satura bajo esa carga.</t>
+        </is>
+      </c>
       <c r="C24" s="55" t="n"/>
       <c r="D24" s="55" t="n"/>
       <c r="E24" s="56" t="n"/>
-      <c r="F24" s="53" t="n"/>
+      <c r="F24" s="53" t="inlineStr">
+        <is>
+          <t>No depender de un endpoint HTTP para telemetría de proceso bajo saturación extrema; instrumentar con un mecanismo fuera de banda (métricas de sistema operativo o del proceso).</t>
+        </is>
+      </c>
       <c r="G24" s="55" t="n"/>
       <c r="H24" s="55" t="n"/>
       <c r="I24" s="55" t="n"/>
@@ -6580,11 +6708,19 @@
           <t>H-05</t>
         </is>
       </c>
-      <c r="B25" s="53" t="n"/>
+      <c r="B25" s="53" t="inlineStr">
+        <is>
+          <t>1.7 GiB de swap seguía en uso tras detener los contenedores ajenos (atribuible a mysqld de sistema y al escritorio), pero el load average bajó a 0.37-0.98 y los resultados coincidieron con la corrida sin contención previa.</t>
+        </is>
+      </c>
       <c r="C25" s="55" t="n"/>
       <c r="D25" s="55" t="n"/>
       <c r="E25" s="56" t="n"/>
-      <c r="F25" s="53" t="n"/>
+      <c r="F25" s="53" t="inlineStr">
+        <is>
+          <t>Para pruebas de estrés reproducibles, monitorear el load average del host como variable de control principal, no solo el swap residual.</t>
+        </is>
+      </c>
       <c r="G25" s="55" t="n"/>
       <c r="H25" s="55" t="n"/>
       <c r="I25" s="55" t="n"/>
@@ -6964,7 +7100,7 @@
     <row r="2" ht="26.15" customHeight="1" s="45">
       <c r="B2" s="46" t="inlineStr">
         <is>
-          <t>CRITERIOS DE ACEPTACIÓN PARA LA ENTREGA</t>
+          <t>CRITERIOS DE ACEPTACIÓN PARA LA ENTREGA · portfolio (codebymike.tech)</t>
         </is>
       </c>
     </row>
@@ -6996,21 +7132,29 @@
     <row r="7" ht="20.15" customHeight="1" s="45">
       <c r="B7" s="40" t="inlineStr">
         <is>
-          <t>Pruebas unitarias aprobadas</t>
+          <t>Pruebas unitarias aprobadas (Vitest)</t>
         </is>
       </c>
       <c r="C7" s="41" t="inlineStr">
         <is>
-          <t>10 de 10</t>
-        </is>
-      </c>
-      <c r="D7" s="42" t="n"/>
-      <c r="E7" s="28" t="n"/>
+          <t>1379 de 1379</t>
+        </is>
+      </c>
+      <c r="D7" s="42" t="inlineStr">
+        <is>
+          <t>1379 de 1379 (413 suites, 0 fallos, 2026-08-31)</t>
+        </is>
+      </c>
+      <c r="E7" s="28" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="20.15" customHeight="1" s="45">
       <c r="B8" s="40" t="inlineStr">
         <is>
-          <t>Cobertura de líneas del paquete service (JaCoCo)</t>
+          <t>Cobertura de líneas de src/lib (v8, `npm run test:coverage`)</t>
         </is>
       </c>
       <c r="C8" s="41" t="inlineStr">
@@ -7018,13 +7162,21 @@
           <t>≥ 80 %</t>
         </is>
       </c>
-      <c r="D8" s="42" t="n"/>
-      <c r="E8" s="28" t="n"/>
+      <c r="D8" s="42" t="inlineStr">
+        <is>
+          <t>71.84 % (3777/5257 líneas)</t>
+        </is>
+      </c>
+      <c r="E8" s="28" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="30.5" customHeight="1" s="45">
       <c r="B9" s="40" t="inlineStr">
         <is>
-          <t>Cobertura de ramas del paquete service (JaCoCo)</t>
+          <t>Cobertura de ramas de src/lib (v8)</t>
         </is>
       </c>
       <c r="C9" s="41" t="inlineStr">
@@ -7032,22 +7184,38 @@
           <t>≥ 70 %</t>
         </is>
       </c>
-      <c r="D9" s="42" t="n"/>
-      <c r="E9" s="28" t="n"/>
+      <c r="D9" s="42" t="inlineStr">
+        <is>
+          <t>65.67 % (2870/4370 ramas)</t>
+        </is>
+      </c>
+      <c r="E9" s="28" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="20.15" customHeight="1" s="45">
       <c r="B10" s="40" t="inlineStr">
         <is>
-          <t>Pruebas de integración aprobadas</t>
+          <t>Pruebas de integración (Playwright e2e) aprobadas</t>
         </is>
       </c>
       <c r="C10" s="41" t="inlineStr">
         <is>
-          <t>12 de 12</t>
-        </is>
-      </c>
-      <c r="D10" s="42" t="n"/>
-      <c r="E10" s="28" t="n"/>
+          <t>48 de 48</t>
+        </is>
+      </c>
+      <c r="D10" s="42" t="inlineStr">
+        <is>
+          <t>44 aprobadas, 1 fallida, 3 bloqueadas en cascada, de 48 (2026-08-31)</t>
+        </is>
+      </c>
+      <c r="E10" s="28" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="20.15" customHeight="1" s="45">
       <c r="B11" s="40" t="inlineStr">
@@ -7060,27 +7228,43 @@
           <t>Sí</t>
         </is>
       </c>
-      <c r="D11" s="42" t="n"/>
-      <c r="E11" s="28" t="n"/>
+      <c r="D11" s="42" t="inlineStr">
+        <is>
+          <t>Pendiente: capa viva del portal (digest) responde 401 en vez de 200 (ver PI-11)</t>
+        </is>
+      </c>
+      <c r="E11" s="28" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="20.15" customHeight="1" s="45">
       <c r="B12" s="40" t="inlineStr">
         <is>
-          <t>Percentil 95 del listado bajo 100 usuarios</t>
+          <t>Percentil 95 de rutas públicas a la carga declarada (25 VUs)</t>
         </is>
       </c>
       <c r="C12" s="41" t="inlineStr">
         <is>
-          <t>≤ 1000 ms</t>
-        </is>
-      </c>
-      <c r="D12" s="42" t="n"/>
-      <c r="E12" s="28" t="n"/>
+          <t>≤ 800 ms</t>
+        </is>
+      </c>
+      <c r="D12" s="42" t="inlineStr">
+        <is>
+          <t>2591 ms (PC-01)</t>
+        </is>
+      </c>
+      <c r="E12" s="28" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="20.15" customHeight="1" s="45">
       <c r="B13" s="40" t="inlineStr">
         <is>
-          <t>Tasa de error bajo carga objetivo</t>
+          <t>Tasa de error bajo la carga declarada (25 VUs)</t>
         </is>
       </c>
       <c r="C13" s="41" t="inlineStr">
@@ -7088,13 +7272,21 @@
           <t>&lt; 1 %</t>
         </is>
       </c>
-      <c r="D13" s="42" t="n"/>
-      <c r="E13" s="28" t="n"/>
+      <c r="D13" s="42" t="inlineStr">
+        <is>
+          <t>0 % (PC-02)</t>
+        </is>
+      </c>
+      <c r="E13" s="28" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="20.15" customHeight="1" s="45">
       <c r="B14" s="40" t="inlineStr">
         <is>
-          <t>Throughput mínimo sostenido</t>
+          <t>Throughput exitoso mínimo sostenido a la carga declarada</t>
         </is>
       </c>
       <c r="C14" s="41" t="inlineStr">
@@ -7102,8 +7294,16 @@
           <t>≥ 60 req/s</t>
         </is>
       </c>
-      <c r="D14" s="42" t="n"/>
-      <c r="E14" s="28" t="n"/>
+      <c r="D14" s="42" t="inlineStr">
+        <is>
+          <t>11.8 req/s (PC-10)</t>
+        </is>
+      </c>
+      <c r="E14" s="28" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="20.15" customHeight="1" s="45">
       <c r="B15" s="40" t="inlineStr">
@@ -7116,8 +7316,16 @@
           <t>Sí</t>
         </is>
       </c>
-      <c r="D15" s="42" t="n"/>
-      <c r="E15" s="28" t="n"/>
+      <c r="D15" s="42" t="inlineStr">
+        <is>
+          <t>Sí: entre 100 y 200 req/s ofrecidos (E2→E3)</t>
+        </is>
+      </c>
+      <c r="E15" s="28" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="20.15" customHeight="1" s="45">
       <c r="B16" s="40" t="inlineStr">
@@ -7130,13 +7338,21 @@
           <t>Sí</t>
         </is>
       </c>
-      <c r="D16" s="42" t="n"/>
-      <c r="E16" s="28" t="n"/>
+      <c r="D16" s="42" t="inlineStr">
+        <is>
+          <t>Sí: 200 req/s ofrecidos, 76.3 % de error (E3, H-01)</t>
+        </is>
+      </c>
+      <c r="E16" s="28" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="20.15" customHeight="1" s="45">
       <c r="B17" s="40" t="inlineStr">
         <is>
-          <t>Recuperación automática tras el estrés</t>
+          <t>Recuperación tras el estrés</t>
         </is>
       </c>
       <c r="C17" s="41" t="inlineStr">
@@ -7144,8 +7360,16 @@
           <t>&lt; 5 min</t>
         </is>
       </c>
-      <c r="D17" s="42" t="n"/>
-      <c r="E17" s="28" t="n"/>
+      <c r="D17" s="42" t="inlineStr">
+        <is>
+          <t>~75-90 s hasta converger por completo (H-02)</t>
+        </is>
+      </c>
+      <c r="E17" s="28" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="20.15" customHeight="1" s="45">
       <c r="B18" s="40" t="inlineStr">
@@ -7158,8 +7382,16 @@
           <t>15 pantallazos</t>
         </is>
       </c>
-      <c r="D18" s="42" t="n"/>
-      <c r="E18" s="28" t="n"/>
+      <c r="D18" s="42" t="inlineStr">
+        <is>
+          <t>Pendiente: corrida automatizada (JSON de vitest/playwright/k6), sin captura manual todavía</t>
+        </is>
+      </c>
+      <c r="E18" s="28" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="20.15" customHeight="1" s="45">
       <c r="B19" s="40" t="inlineStr">
@@ -7172,8 +7404,16 @@
           <t>Sí</t>
         </is>
       </c>
-      <c r="D19" s="42" t="n"/>
-      <c r="E19" s="28" t="n"/>
+      <c r="D19" s="42" t="inlineStr">
+        <is>
+          <t>Sí, en cada hoja (M1-M4) y en esta</t>
+        </is>
+      </c>
+      <c r="E19" s="28" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="B21" s="1" t="inlineStr">
@@ -7205,7 +7445,11 @@
           <t>Responsable de las pruebas</t>
         </is>
       </c>
-      <c r="C24" s="10" t="n"/>
+      <c r="C24" s="10" t="inlineStr">
+        <is>
+          <t>Mike (@mikerb95)</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="B25" s="9" t="inlineStr">
@@ -7213,7 +7457,11 @@
           <t>Instructor</t>
         </is>
       </c>
-      <c r="C25" s="10" t="n"/>
+      <c r="C25" s="10" t="inlineStr">
+        <is>
+          <t>N/A — proyecto de práctica independiente, sin instructor asignado en esta iteración</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="B26" s="9" t="inlineStr">
@@ -7221,7 +7469,11 @@
           <t>Fecha de la evaluación</t>
         </is>
       </c>
-      <c r="C26" s="10" t="n"/>
+      <c r="C26" s="10" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="3">

</xml_diff>